<commit_message>
update my daily log
</commit_message>
<xml_diff>
--- a/1234567.xlsx
+++ b/1234567.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5731650e8b717ef2/Desktop/CAP776/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="94" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{53FEA915-4809-4A3B-A27A-49D90D30E963}"/>
+  <xr:revisionPtr revIDLastSave="105" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1B9208CB-0313-4BD6-A1A6-EC4703C8D60E}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="66">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -230,6 +230,9 @@
   </si>
   <si>
     <t>I gave Ca very well</t>
+  </si>
+  <si>
+    <t>Neutral</t>
   </si>
 </sst>
 </file>
@@ -1300,25 +1303,47 @@
       <c r="N11" s="16"/>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A12" s="12"/>
-      <c r="B12" s="13"/>
-      <c r="C12" s="13"/>
-      <c r="D12" s="13"/>
-      <c r="E12" s="13"/>
-      <c r="F12" s="13"/>
-      <c r="G12" s="13"/>
-      <c r="H12" s="13"/>
-      <c r="I12" s="14" t="str">
+      <c r="A12" s="12">
+        <v>46275</v>
+      </c>
+      <c r="B12" s="13">
+        <v>360</v>
+      </c>
+      <c r="C12" s="13">
+        <v>60</v>
+      </c>
+      <c r="D12" s="13">
+        <v>180</v>
+      </c>
+      <c r="E12" s="13">
+        <v>60</v>
+      </c>
+      <c r="F12" s="13">
+        <v>100</v>
+      </c>
+      <c r="G12" s="13">
+        <v>2</v>
+      </c>
+      <c r="H12" s="13">
+        <v>200</v>
+      </c>
+      <c r="I12" s="14">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J12" s="14" t="str">
+        <v>960</v>
+      </c>
+      <c r="J12" s="14">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K12" s="15"/>
-      <c r="L12" s="15"/>
-      <c r="M12" s="15"/>
+        <v>480</v>
+      </c>
+      <c r="K12" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="L12" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="M12" s="15" t="s">
+        <v>51</v>
+      </c>
       <c r="N12" s="16"/>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.35">

</xml_diff>